<commit_message>
[SKA]-Added Start and End date in pricelist import script
</commit_message>
<xml_diff>
--- a/baur_pricelist_import/static/sample/pricelist_import_sample.xlsx
+++ b/baur_pricelist_import/static/sample/pricelist_import_sample.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +48,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,6 +440,16 @@
           <t>Price</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>End Date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -455,6 +468,12 @@
       <c r="D2" t="n">
         <v>19.99</v>
       </c>
+      <c r="E2" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>46022</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -473,6 +492,12 @@
       <c r="D3" t="n">
         <v>17.5</v>
       </c>
+      <c r="E3" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>46022</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -490,6 +515,12 @@
       </c>
       <c r="D4" t="n">
         <v>8</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>46022</v>
       </c>
     </row>
   </sheetData>

</xml_diff>